<commit_message>
Complete restaurant budget review and guard invalid thresholds [skip social]
</commit_message>
<xml_diff>
--- a/public/downloads/restaurant-monthly-budget-template.xlsx
+++ b/public/downloads/restaurant-monthly-budget-template.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monthly Budget" sheetId="1" r:id="R15f3a75823554ba5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monthly Budget" sheetId="1" r:id="R0a89cbca97bc4b12"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -17,7 +17,7 @@
     <x:numFmt numFmtId="200" formatCode="&quot;$&quot;#,##0;(&quot;$&quot;#,##0);-"/>
     <x:numFmt numFmtId="201" formatCode="0.0%"/>
   </x:numFmts>
-  <x:fonts count="5">
+  <x:fonts count="6">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -42,6 +42,11 @@
     <x:font>
       <x:sz val="10"/>
       <x:color rgb="FF1750A1"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:color rgb="FF243144"/>
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
@@ -79,7 +84,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="15">
+  <x:cellXfs count="22">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -95,6 +100,27 @@
     <x:xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="200" fontId="1" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="201" fontId="1" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="1" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="1" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="1" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="1" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -582,34 +608,34 @@
       <x:c r="E19" s="1"/>
     </x:row>
     <x:row r="20">
-      <x:c r="A20" s="12" t="str">
+      <x:c r="A20" s="19" t="str">
         <x:v>Contribution margin</x:v>
       </x:c>
-      <x:c r="B20" s="14" t="n">
-        <x:f>IFERROR(B11/B8,0)</x:f>
+      <x:c r="B20" s="20" t="n">
+        <x:f>IF(COUNT(B6:B7,B9:B10)&lt;&gt;4,"Complete inputs",IF(MIN(B6:B7,B9:B10)&lt;0,"Check inputs",IF(B8&lt;=0,"No sales",B11/B8)))</x:f>
         <x:v>0.7</x:v>
       </x:c>
-      <x:c r="C20" s="14" t="n">
-        <x:f>IFERROR(C11/C8,0)</x:f>
+      <x:c r="C20" s="20" t="n">
+        <x:f>IF(COUNT(C6:C7,C9:C10)&lt;&gt;4,"Complete inputs",IF(MIN(C6:C7,C9:C10)&lt;0,"Check inputs",IF(C8&lt;=0,"No sales",C11/C8)))</x:f>
         <x:v>0.6719298245614035</x:v>
       </x:c>
-      <x:c r="D20" s="13"/>
+      <x:c r="D20" s="21"/>
       <x:c r="E20" s="1"/>
     </x:row>
-    <x:row r="21">
-      <x:c r="A21" s="12" t="str">
+    <x:row r="21" ht="46" customHeight="1">
+      <x:c r="A21" s="19" t="str">
         <x:v>Break-even sales</x:v>
       </x:c>
-      <x:c r="B21" s="13" t="n">
-        <x:f>IFERROR(SUM(B12:B18)/B20,0)</x:f>
+      <x:c r="B21" s="21" t="n">
+        <x:f>IF(COUNT(B6:B7,B9:B10,B12:B18)&lt;&gt;11,"Complete inputs",IF(MIN(B6:B7,B9:B10,B12:B18)&lt;0,"Check inputs",IF(B8&lt;=0,"No sales",IF(B11&lt;=0,"No positive contribution",SUM(B12:B18)/(B11/B8)))))</x:f>
         <x:v>43142.857142857145</x:v>
       </x:c>
-      <x:c r="C21" s="13" t="n">
-        <x:f>IFERROR(SUM(C12:C18)/C20,0)</x:f>
+      <x:c r="C21" s="21" t="n">
+        <x:f>IF(COUNT(C6:C7,C9:C10,C12:C18)&lt;&gt;11,"Complete inputs",IF(MIN(C6:C7,C9:C10,C12:C18)&lt;0,"Check inputs",IF(C8&lt;=0,"No sales",IF(C11&lt;=0,"No positive contribution",SUM(C12:C18)/(C11/C8)))))</x:f>
         <x:v>46284.5953002611</x:v>
       </x:c>
-      <x:c r="D21" s="13" t="n">
-        <x:f>C21-B21</x:f>
+      <x:c r="D21" s="21" t="n">
+        <x:f>IF(AND(ISNUMBER(B21),ISNUMBER(C21)),C21-B21,"Not comparable")</x:f>
         <x:v>3141.7381574039537</x:v>
       </x:c>
       <x:c r="E21" s="1"/>
@@ -646,43 +672,43 @@
       <x:c r="D25" s="1"/>
       <x:c r="E25" s="1"/>
     </x:row>
-    <x:row r="26">
-      <x:c r="A26" s="1" t="str">
-        <x:v>Method: contribution margin and fixed/variable separation per SBA.</x:v>
-      </x:c>
-      <x:c r="B26" s="1" t="str">
-        <x:v>https://www.sba.gov/business-guide/plan-your-business/calculate-your-startup-costs/break-even-point</x:v>
-      </x:c>
-      <x:c r="C26" s="1"/>
-      <x:c r="D26" s="1"/>
+    <x:row r="26" ht="26" customHeight="1">
+      <x:c r="A26" s="17" t="str">
+        <x:v>Method: contribution margin and fixed/variable separation, SBA. https://www.sba.gov/business-guide/plan-your-business/calculate-your-startup-costs/break-even-point</x:v>
+      </x:c>
+      <x:c r="B26" s="17"/>
+      <x:c r="C26" s="17"/>
+      <x:c r="D26" s="17"/>
       <x:c r="E26" s="1"/>
     </x:row>
-    <x:row r="27">
-      <x:c r="A27" s="1"/>
-      <x:c r="B27" s="1"/>
-      <x:c r="C27" s="1"/>
-      <x:c r="D27" s="1"/>
+    <x:row r="27" ht="26" customHeight="1">
+      <x:c r="A27" s="17"/>
+      <x:c r="B27" s="17"/>
+      <x:c r="C27" s="17"/>
+      <x:c r="D27" s="17"/>
       <x:c r="E27" s="1"/>
     </x:row>
     <x:row r="28">
-      <x:c r="A28" s="1"/>
-      <x:c r="B28" s="1"/>
-      <x:c r="C28" s="1"/>
-      <x:c r="D28" s="1"/>
+      <x:c r="A28" s="18" t="str">
+        <x:v>Break-even needs positive sales and contribution. Complete inputs = missing/nonnumeric amount; Check inputs = negative amount. Enter 0 only for a cost or sales line that is genuinely zero. No positive contribution is not a zero-sales target.</x:v>
+      </x:c>
+      <x:c r="B28" s="18"/>
+      <x:c r="C28" s="18"/>
+      <x:c r="D28" s="18"/>
       <x:c r="E28" s="1"/>
     </x:row>
     <x:row r="29">
-      <x:c r="A29" s="1"/>
-      <x:c r="B29" s="1"/>
-      <x:c r="C29" s="1"/>
-      <x:c r="D29" s="1"/>
+      <x:c r="A29" s="18"/>
+      <x:c r="B29" s="18"/>
+      <x:c r="C29" s="18"/>
+      <x:c r="D29" s="18"/>
       <x:c r="E29" s="1"/>
     </x:row>
     <x:row r="30">
-      <x:c r="A30" s="1"/>
-      <x:c r="B30" s="1"/>
-      <x:c r="C30" s="1"/>
-      <x:c r="D30" s="1"/>
+      <x:c r="A30" s="18"/>
+      <x:c r="B30" s="18"/>
+      <x:c r="C30" s="18"/>
+      <x:c r="D30" s="18"/>
       <x:c r="E30" s="1"/>
     </x:row>
     <x:row r="31">
@@ -756,6 +782,10 @@
       <x:c r="E40" s="1"/>
     </x:row>
   </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A28:D30"/>
+    <x:mergeCell ref="A26:D27"/>
+  </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
 </file>
</xml_diff>